<commit_message>
QC & FIX  - agregat penduduk
</commit_message>
<xml_diff>
--- a/public/format_file_excel_import/penduduk_pekerjaan.xlsx
+++ b/public/format_file_excel_import/penduduk_pekerjaan.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10309"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ariesyarwani/Documents/format excel import/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\Rumah data 2.0\public\format_file_excel_import\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09278BF0-C8CB-8849-85B4-0BADE79A954F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{180AA9BB-B3C4-490C-98DD-B92558633BEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1080" yWindow="1240" windowWidth="27640" windowHeight="16760" xr2:uid="{9F0C61F8-DFF9-114A-8F8C-91ECB181F7CD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9F0C61F8-DFF9-114A-8F8C-91ECB181F7CD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -485,30 +485,12 @@
     <t>perawat_p</t>
   </si>
   <si>
-    <t>apotek_l</t>
-  </si>
-  <si>
-    <t>apotek_p</t>
-  </si>
-  <si>
     <t>psikiater_psikolog_l</t>
   </si>
   <si>
     <t>psikiater_psikolog_p</t>
   </si>
   <si>
-    <t>penyiara_televisi_l</t>
-  </si>
-  <si>
-    <t>penyiara_televisi_p</t>
-  </si>
-  <si>
-    <t>penyiara_radio_l</t>
-  </si>
-  <si>
-    <t>penyiara_radio_p</t>
-  </si>
-  <si>
     <t>pelaut_l</t>
   </si>
   <si>
@@ -611,12 +593,6 @@
     <t>operator_p</t>
   </si>
   <si>
-    <t>pekerja_pengolahan_krajinan_l</t>
-  </si>
-  <si>
-    <t>pekerja_pengolahan_krajinan_p</t>
-  </si>
-  <si>
     <t>teknisi_l</t>
   </si>
   <si>
@@ -633,13 +609,37 @@
   </si>
   <si>
     <t>pekerjaan_lainnya_p</t>
+  </si>
+  <si>
+    <t>apoteker_l</t>
+  </si>
+  <si>
+    <t>apoteker_p</t>
+  </si>
+  <si>
+    <t>penyiar_televisi_l</t>
+  </si>
+  <si>
+    <t>penyiar_televisi_p</t>
+  </si>
+  <si>
+    <t>penyiar_radio_l</t>
+  </si>
+  <si>
+    <t>penyiar_radio_p</t>
+  </si>
+  <si>
+    <t>pekerja_pengolahan_kerajinan_l</t>
+  </si>
+  <si>
+    <t>pekerja_pengolahan_kerajinan_p</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -653,16 +653,30 @@
       <name val="Menlo"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor theme="4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -670,18 +684,59 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -714,10 +769,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6D6ED365-FED1-7447-8572-39D953C49024}" name="Table1" displayName="Table1" ref="A1:GQ2" insertRow="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6D6ED365-FED1-7447-8572-39D953C49024}" name="Table1" displayName="Table1" ref="A1:GQ2" insertRow="1" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="1">
   <autoFilter ref="A1:GQ2" xr:uid="{6D6ED365-FED1-7447-8572-39D953C49024}"/>
   <tableColumns count="199">
-    <tableColumn id="1" xr3:uid="{345D1603-B35C-1C46-9376-47E0FA657326}" name="kode_wilayah" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{345D1603-B35C-1C46-9376-47E0FA657326}" name="kode_wilayah" dataDxfId="2"/>
     <tableColumn id="2" xr3:uid="{08A23DFB-0653-4F40-9EF0-93692889FC50}" name="belum_tidak_bekerja_l"/>
     <tableColumn id="3" xr3:uid="{729604AD-7B07-4A47-B6D9-EDF35222846D}" name="belum_tidak_bekerja_p"/>
     <tableColumn id="4" xr3:uid="{32C6062E-6C13-534D-8037-72AE2940FAAD}" name="mengurus_rumah_tangga_l"/>
@@ -866,14 +921,14 @@
     <tableColumn id="147" xr3:uid="{0E154EF8-1134-8B44-AADB-D6338C758F7C}" name="bidan_p"/>
     <tableColumn id="148" xr3:uid="{B170464D-64E9-F24C-9772-16D99F991E8C}" name="perawat_l"/>
     <tableColumn id="149" xr3:uid="{0BE954E5-43F0-3C48-9763-98CCD9A253EC}" name="perawat_p"/>
-    <tableColumn id="150" xr3:uid="{3B8CD2A9-4DBE-4740-8988-DDCDC1B49277}" name="apotek_l"/>
-    <tableColumn id="151" xr3:uid="{55D2544B-4114-F644-BEEA-FB4FFD85A7DC}" name="apotek_p"/>
+    <tableColumn id="150" xr3:uid="{3B8CD2A9-4DBE-4740-8988-DDCDC1B49277}" name="apoteker_l"/>
+    <tableColumn id="151" xr3:uid="{55D2544B-4114-F644-BEEA-FB4FFD85A7DC}" name="apoteker_p"/>
     <tableColumn id="152" xr3:uid="{890B2171-31FF-5F44-A853-5EB031BEE5F1}" name="psikiater_psikolog_l"/>
     <tableColumn id="153" xr3:uid="{997A8167-D7D9-3A4E-9BDD-A73359E5C116}" name="psikiater_psikolog_p"/>
-    <tableColumn id="154" xr3:uid="{167AC58A-3B3B-AD4A-A418-0F7045CCE44C}" name="penyiara_televisi_l"/>
-    <tableColumn id="155" xr3:uid="{99038E0D-9011-A747-83B5-47BEDDC2D8DB}" name="penyiara_televisi_p"/>
-    <tableColumn id="156" xr3:uid="{151FB6F7-DA79-0D42-BC55-AFAAF804F269}" name="penyiara_radio_l"/>
-    <tableColumn id="157" xr3:uid="{D8D83E16-B2E3-3347-A167-FA276E49E333}" name="penyiara_radio_p"/>
+    <tableColumn id="154" xr3:uid="{167AC58A-3B3B-AD4A-A418-0F7045CCE44C}" name="penyiar_televisi_l"/>
+    <tableColumn id="155" xr3:uid="{99038E0D-9011-A747-83B5-47BEDDC2D8DB}" name="penyiar_televisi_p"/>
+    <tableColumn id="156" xr3:uid="{151FB6F7-DA79-0D42-BC55-AFAAF804F269}" name="penyiar_radio_l"/>
+    <tableColumn id="157" xr3:uid="{D8D83E16-B2E3-3347-A167-FA276E49E333}" name="penyiar_radio_p"/>
     <tableColumn id="158" xr3:uid="{21AECABF-C6AD-724A-B8DF-284A82B46953}" name="pelaut_l"/>
     <tableColumn id="159" xr3:uid="{6290290F-C729-044D-AFC4-86EBCA9C5A31}" name="pelaut_p"/>
     <tableColumn id="160" xr3:uid="{2BFE5278-D223-2B49-8DF5-E29EADF2BB8B}" name="peneliti_l"/>
@@ -908,8 +963,8 @@
     <tableColumn id="189" xr3:uid="{696D48D1-B52C-ED4C-AF85-877662156C8B}" name="tenaga_tata_usaha_p"/>
     <tableColumn id="190" xr3:uid="{5305D929-B508-014A-9C1C-F0C3BCFD0762}" name="operator_l"/>
     <tableColumn id="191" xr3:uid="{8DDCC566-91A3-874C-85E3-67928768E57A}" name="operator_p"/>
-    <tableColumn id="192" xr3:uid="{C139AC47-CA6C-0B42-BBCF-2D9583E47146}" name="pekerja_pengolahan_krajinan_l"/>
-    <tableColumn id="193" xr3:uid="{D831925F-0341-B248-A1EA-9C1A6FB51B2F}" name="pekerja_pengolahan_krajinan_p"/>
+    <tableColumn id="192" xr3:uid="{C139AC47-CA6C-0B42-BBCF-2D9583E47146}" name="pekerja_pengolahan_kerajinan_l"/>
+    <tableColumn id="193" xr3:uid="{D831925F-0341-B248-A1EA-9C1A6FB51B2F}" name="pekerja_pengolahan_kerajinan_p"/>
     <tableColumn id="194" xr3:uid="{61C506F1-2B8B-FC40-82C2-C80DFDEF03CC}" name="teknisi_l"/>
     <tableColumn id="195" xr3:uid="{509BFF65-4EF6-4340-969F-BE01BEB66216}" name="teknisi_p"/>
     <tableColumn id="196" xr3:uid="{FF834328-DE44-CC4F-B5C8-53D15BA71EFD}" name="asisten_ahli_l"/>
@@ -1239,1367 +1294,1367 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{078D12A0-4C6E-E740-89EE-DEA1F076E528}">
   <dimension ref="A1:GQ199"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="14.5" customWidth="1"/>
+    <col min="1" max="1" width="14.44140625" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="3" max="3" width="22.5" customWidth="1"/>
-    <col min="4" max="4" width="25.83203125" customWidth="1"/>
+    <col min="3" max="3" width="22.44140625" customWidth="1"/>
+    <col min="4" max="4" width="25.77734375" customWidth="1"/>
     <col min="5" max="5" width="26.33203125" customWidth="1"/>
-    <col min="6" max="6" width="20.83203125" customWidth="1"/>
+    <col min="6" max="6" width="20.77734375" customWidth="1"/>
     <col min="7" max="7" width="21.33203125" customWidth="1"/>
     <col min="8" max="8" width="13.33203125" customWidth="1"/>
-    <col min="9" max="9" width="13.83203125" customWidth="1"/>
-    <col min="10" max="10" width="25.83203125" customWidth="1"/>
+    <col min="9" max="9" width="13.77734375" customWidth="1"/>
+    <col min="10" max="10" width="25.77734375" customWidth="1"/>
     <col min="11" max="11" width="26.33203125" customWidth="1"/>
-    <col min="12" max="12" width="30.5" customWidth="1"/>
+    <col min="12" max="12" width="30.44140625" customWidth="1"/>
     <col min="13" max="13" width="31" customWidth="1"/>
-    <col min="14" max="14" width="19.83203125" customWidth="1"/>
+    <col min="14" max="14" width="19.77734375" customWidth="1"/>
     <col min="15" max="15" width="20.33203125" customWidth="1"/>
-    <col min="16" max="16" width="15.5" customWidth="1"/>
+    <col min="16" max="16" width="15.44140625" customWidth="1"/>
     <col min="17" max="17" width="16" customWidth="1"/>
-    <col min="18" max="18" width="17.83203125" customWidth="1"/>
+    <col min="18" max="18" width="17.77734375" customWidth="1"/>
     <col min="19" max="19" width="18.33203125" customWidth="1"/>
-    <col min="20" max="20" width="12.1640625" customWidth="1"/>
+    <col min="20" max="20" width="12.109375" customWidth="1"/>
     <col min="21" max="21" width="12.6640625" customWidth="1"/>
-    <col min="22" max="22" width="20.1640625" customWidth="1"/>
+    <col min="22" max="22" width="20.109375" customWidth="1"/>
     <col min="23" max="23" width="20.6640625" customWidth="1"/>
-    <col min="24" max="24" width="11.1640625" customWidth="1"/>
+    <col min="24" max="24" width="11.109375" customWidth="1"/>
     <col min="25" max="25" width="11.6640625" customWidth="1"/>
     <col min="26" max="26" width="13.6640625" customWidth="1"/>
-    <col min="27" max="27" width="14.1640625" customWidth="1"/>
+    <col min="27" max="27" width="14.109375" customWidth="1"/>
     <col min="28" max="28" width="15" customWidth="1"/>
-    <col min="29" max="29" width="15.5" customWidth="1"/>
-    <col min="30" max="30" width="19.5" customWidth="1"/>
+    <col min="29" max="29" width="15.44140625" customWidth="1"/>
+    <col min="30" max="30" width="19.44140625" customWidth="1"/>
     <col min="31" max="31" width="20" customWidth="1"/>
-    <col min="32" max="32" width="18.1640625" customWidth="1"/>
+    <col min="32" max="32" width="18.109375" customWidth="1"/>
     <col min="33" max="33" width="18.6640625" customWidth="1"/>
-    <col min="34" max="34" width="18.1640625" customWidth="1"/>
+    <col min="34" max="34" width="18.109375" customWidth="1"/>
     <col min="35" max="35" width="18.6640625" customWidth="1"/>
-    <col min="36" max="36" width="19.83203125" customWidth="1"/>
+    <col min="36" max="36" width="19.77734375" customWidth="1"/>
     <col min="37" max="37" width="20.33203125" customWidth="1"/>
-    <col min="38" max="38" width="20.83203125" customWidth="1"/>
+    <col min="38" max="38" width="20.77734375" customWidth="1"/>
     <col min="39" max="39" width="21.33203125" customWidth="1"/>
     <col min="40" max="40" width="24" customWidth="1"/>
-    <col min="41" max="41" width="24.5" customWidth="1"/>
+    <col min="41" max="41" width="24.44140625" customWidth="1"/>
     <col min="42" max="42" width="25.6640625" customWidth="1"/>
-    <col min="43" max="43" width="26.1640625" customWidth="1"/>
+    <col min="43" max="43" width="26.109375" customWidth="1"/>
     <col min="44" max="44" width="19.6640625" customWidth="1"/>
-    <col min="45" max="45" width="20.1640625" customWidth="1"/>
-    <col min="46" max="46" width="25.83203125" customWidth="1"/>
+    <col min="45" max="45" width="20.109375" customWidth="1"/>
+    <col min="46" max="46" width="25.77734375" customWidth="1"/>
     <col min="47" max="47" width="26.33203125" customWidth="1"/>
     <col min="48" max="48" width="16" customWidth="1"/>
-    <col min="49" max="49" width="16.5" customWidth="1"/>
-    <col min="50" max="50" width="16.1640625" customWidth="1"/>
+    <col min="49" max="49" width="16.44140625" customWidth="1"/>
+    <col min="50" max="50" width="16.109375" customWidth="1"/>
     <col min="51" max="51" width="16.6640625" customWidth="1"/>
     <col min="52" max="52" width="15" customWidth="1"/>
-    <col min="53" max="53" width="15.5" customWidth="1"/>
-    <col min="54" max="54" width="15.1640625" customWidth="1"/>
+    <col min="53" max="53" width="15.44140625" customWidth="1"/>
+    <col min="54" max="54" width="15.109375" customWidth="1"/>
     <col min="55" max="55" width="15.6640625" customWidth="1"/>
     <col min="56" max="56" width="20.33203125" customWidth="1"/>
-    <col min="57" max="57" width="20.83203125" customWidth="1"/>
-    <col min="58" max="58" width="24.5" customWidth="1"/>
+    <col min="57" max="57" width="20.77734375" customWidth="1"/>
+    <col min="58" max="58" width="24.44140625" customWidth="1"/>
     <col min="59" max="59" width="25" customWidth="1"/>
     <col min="60" max="60" width="15" customWidth="1"/>
-    <col min="61" max="61" width="15.5" customWidth="1"/>
+    <col min="61" max="61" width="15.44140625" customWidth="1"/>
     <col min="62" max="62" width="14.33203125" customWidth="1"/>
-    <col min="63" max="63" width="14.83203125" customWidth="1"/>
-    <col min="64" max="64" width="14.5" customWidth="1"/>
+    <col min="63" max="63" width="14.77734375" customWidth="1"/>
+    <col min="64" max="64" width="14.44140625" customWidth="1"/>
     <col min="65" max="65" width="15" customWidth="1"/>
     <col min="66" max="66" width="17.33203125" customWidth="1"/>
-    <col min="67" max="67" width="17.83203125" customWidth="1"/>
+    <col min="67" max="67" width="17.77734375" customWidth="1"/>
     <col min="68" max="68" width="17.33203125" customWidth="1"/>
-    <col min="69" max="69" width="17.83203125" customWidth="1"/>
+    <col min="69" max="69" width="17.77734375" customWidth="1"/>
     <col min="70" max="70" width="12" customWidth="1"/>
-    <col min="71" max="71" width="12.5" customWidth="1"/>
+    <col min="71" max="71" width="12.44140625" customWidth="1"/>
     <col min="72" max="72" width="12" customWidth="1"/>
-    <col min="73" max="73" width="12.5" customWidth="1"/>
+    <col min="73" max="73" width="12.44140625" customWidth="1"/>
     <col min="78" max="78" width="20.33203125" customWidth="1"/>
-    <col min="79" max="79" width="20.83203125" customWidth="1"/>
+    <col min="79" max="79" width="20.77734375" customWidth="1"/>
     <col min="80" max="80" width="15.33203125" customWidth="1"/>
-    <col min="81" max="81" width="15.83203125" customWidth="1"/>
-    <col min="82" max="82" width="16.1640625" customWidth="1"/>
+    <col min="81" max="81" width="15.77734375" customWidth="1"/>
+    <col min="82" max="82" width="16.109375" customWidth="1"/>
     <col min="83" max="83" width="16.6640625" customWidth="1"/>
-    <col min="84" max="84" width="11.5" customWidth="1"/>
+    <col min="84" max="84" width="11.44140625" customWidth="1"/>
     <col min="85" max="85" width="12" customWidth="1"/>
-    <col min="88" max="88" width="12.83203125" customWidth="1"/>
+    <col min="88" max="88" width="12.77734375" customWidth="1"/>
     <col min="89" max="89" width="13.33203125" customWidth="1"/>
-    <col min="90" max="90" width="18.83203125" customWidth="1"/>
+    <col min="90" max="90" width="18.77734375" customWidth="1"/>
     <col min="91" max="91" width="19.33203125" customWidth="1"/>
-    <col min="92" max="92" width="14.5" customWidth="1"/>
+    <col min="92" max="92" width="14.44140625" customWidth="1"/>
     <col min="93" max="93" width="15" customWidth="1"/>
     <col min="94" max="94" width="18" customWidth="1"/>
-    <col min="95" max="95" width="18.5" customWidth="1"/>
+    <col min="95" max="95" width="18.44140625" customWidth="1"/>
     <col min="96" max="96" width="17" customWidth="1"/>
-    <col min="97" max="97" width="17.5" customWidth="1"/>
+    <col min="97" max="97" width="17.44140625" customWidth="1"/>
     <col min="98" max="98" width="17.33203125" customWidth="1"/>
-    <col min="99" max="99" width="17.83203125" customWidth="1"/>
+    <col min="99" max="99" width="17.77734375" customWidth="1"/>
     <col min="100" max="100" width="15.33203125" customWidth="1"/>
-    <col min="101" max="101" width="15.83203125" customWidth="1"/>
+    <col min="101" max="101" width="15.77734375" customWidth="1"/>
     <col min="102" max="102" width="12" customWidth="1"/>
-    <col min="103" max="103" width="12.5" customWidth="1"/>
-    <col min="104" max="104" width="17.1640625" customWidth="1"/>
+    <col min="103" max="103" width="12.44140625" customWidth="1"/>
+    <col min="104" max="104" width="17.109375" customWidth="1"/>
     <col min="105" max="105" width="17.6640625" customWidth="1"/>
-    <col min="106" max="106" width="30.83203125" customWidth="1"/>
+    <col min="106" max="106" width="30.77734375" customWidth="1"/>
     <col min="107" max="107" width="31.33203125" customWidth="1"/>
-    <col min="108" max="108" width="29.83203125" customWidth="1"/>
+    <col min="108" max="108" width="29.77734375" customWidth="1"/>
     <col min="109" max="109" width="30.33203125" customWidth="1"/>
     <col min="110" max="110" width="14" customWidth="1"/>
-    <col min="111" max="111" width="14.83203125" customWidth="1"/>
-    <col min="112" max="112" width="12.1640625" customWidth="1"/>
+    <col min="111" max="111" width="14.77734375" customWidth="1"/>
+    <col min="112" max="112" width="12.109375" customWidth="1"/>
     <col min="113" max="113" width="12.6640625" customWidth="1"/>
     <col min="114" max="114" width="17.33203125" customWidth="1"/>
-    <col min="115" max="115" width="17.83203125" customWidth="1"/>
-    <col min="118" max="118" width="15.1640625" customWidth="1"/>
+    <col min="115" max="115" width="17.77734375" customWidth="1"/>
+    <col min="118" max="118" width="15.109375" customWidth="1"/>
     <col min="119" max="119" width="15.6640625" customWidth="1"/>
-    <col min="120" max="120" width="11.83203125" customWidth="1"/>
+    <col min="120" max="120" width="11.77734375" customWidth="1"/>
     <col min="121" max="121" width="12.33203125" customWidth="1"/>
     <col min="122" max="122" width="17" customWidth="1"/>
-    <col min="123" max="123" width="17.5" customWidth="1"/>
-    <col min="124" max="124" width="20.5" customWidth="1"/>
+    <col min="123" max="123" width="17.44140625" customWidth="1"/>
+    <col min="124" max="124" width="20.44140625" customWidth="1"/>
     <col min="125" max="125" width="21" customWidth="1"/>
     <col min="126" max="126" width="24.33203125" customWidth="1"/>
-    <col min="127" max="127" width="24.83203125" customWidth="1"/>
-    <col min="134" max="134" width="13.5" customWidth="1"/>
+    <col min="127" max="127" width="24.77734375" customWidth="1"/>
+    <col min="134" max="134" width="13.44140625" customWidth="1"/>
     <col min="135" max="135" width="14" customWidth="1"/>
-    <col min="137" max="137" width="11.1640625" customWidth="1"/>
-    <col min="139" max="139" width="11.1640625" customWidth="1"/>
-    <col min="140" max="140" width="11.5" customWidth="1"/>
+    <col min="137" max="137" width="11.109375" customWidth="1"/>
+    <col min="139" max="139" width="11.109375" customWidth="1"/>
+    <col min="140" max="140" width="11.44140625" customWidth="1"/>
     <col min="141" max="141" width="12" customWidth="1"/>
     <col min="142" max="142" width="13" customWidth="1"/>
-    <col min="143" max="143" width="13.5" customWidth="1"/>
-    <col min="148" max="148" width="11.5" customWidth="1"/>
+    <col min="143" max="143" width="13.44140625" customWidth="1"/>
+    <col min="148" max="148" width="11.44140625" customWidth="1"/>
     <col min="149" max="149" width="12" customWidth="1"/>
     <col min="151" max="151" width="11" customWidth="1"/>
     <col min="152" max="152" width="20" customWidth="1"/>
-    <col min="153" max="153" width="20.5" customWidth="1"/>
+    <col min="153" max="153" width="20.44140625" customWidth="1"/>
     <col min="154" max="154" width="18.6640625" customWidth="1"/>
-    <col min="155" max="155" width="19.1640625" customWidth="1"/>
-    <col min="156" max="156" width="16.83203125" customWidth="1"/>
+    <col min="155" max="155" width="19.109375" customWidth="1"/>
+    <col min="156" max="156" width="16.77734375" customWidth="1"/>
     <col min="157" max="157" width="17.33203125" customWidth="1"/>
     <col min="160" max="160" width="11" customWidth="1"/>
-    <col min="161" max="161" width="11.5" customWidth="1"/>
+    <col min="161" max="161" width="11.44140625" customWidth="1"/>
     <col min="165" max="165" width="11.33203125" customWidth="1"/>
     <col min="166" max="166" width="14.33203125" customWidth="1"/>
-    <col min="167" max="167" width="14.83203125" customWidth="1"/>
-    <col min="168" max="168" width="12.83203125" customWidth="1"/>
+    <col min="167" max="167" width="14.77734375" customWidth="1"/>
+    <col min="168" max="168" width="12.77734375" customWidth="1"/>
     <col min="169" max="169" width="13.33203125" customWidth="1"/>
     <col min="170" max="170" width="18" customWidth="1"/>
-    <col min="171" max="171" width="18.5" customWidth="1"/>
-    <col min="172" max="172" width="15.1640625" customWidth="1"/>
+    <col min="171" max="171" width="18.44140625" customWidth="1"/>
+    <col min="172" max="172" width="15.109375" customWidth="1"/>
     <col min="173" max="173" width="15.6640625" customWidth="1"/>
-    <col min="174" max="174" width="20.83203125" customWidth="1"/>
+    <col min="174" max="174" width="20.77734375" customWidth="1"/>
     <col min="175" max="175" width="21.33203125" customWidth="1"/>
     <col min="176" max="176" width="14.33203125" customWidth="1"/>
-    <col min="177" max="177" width="14.83203125" customWidth="1"/>
+    <col min="177" max="177" width="14.77734375" customWidth="1"/>
     <col min="178" max="178" width="31.6640625" customWidth="1"/>
-    <col min="179" max="179" width="32.1640625" customWidth="1"/>
+    <col min="179" max="179" width="32.109375" customWidth="1"/>
     <col min="186" max="186" width="11.6640625" customWidth="1"/>
-    <col min="187" max="187" width="12.1640625" customWidth="1"/>
-    <col min="188" max="188" width="20.5" customWidth="1"/>
+    <col min="187" max="187" width="12.109375" customWidth="1"/>
+    <col min="188" max="188" width="20.44140625" customWidth="1"/>
     <col min="189" max="189" width="21" customWidth="1"/>
-    <col min="190" max="190" width="11.83203125" customWidth="1"/>
+    <col min="190" max="190" width="11.77734375" customWidth="1"/>
     <col min="191" max="191" width="12.33203125" customWidth="1"/>
-    <col min="192" max="192" width="28.83203125" customWidth="1"/>
+    <col min="192" max="192" width="28.77734375" customWidth="1"/>
     <col min="193" max="193" width="29.33203125" customWidth="1"/>
     <col min="195" max="195" width="11" customWidth="1"/>
-    <col min="196" max="196" width="14.83203125" customWidth="1"/>
+    <col min="196" max="196" width="14.77734375" customWidth="1"/>
     <col min="197" max="197" width="15.33203125" customWidth="1"/>
     <col min="198" max="198" width="19.6640625" customWidth="1"/>
-    <col min="199" max="199" width="20.1640625" customWidth="1"/>
+    <col min="199" max="199" width="20.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:199" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+    <row r="1" spans="1:199" ht="15.75">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AB1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AC1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AD1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AE1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AF1" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AG1" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AH1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AI1" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AJ1" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AK1" t="s">
+      <c r="AK1" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="AL1" t="s">
+      <c r="AL1" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="AM1" t="s">
+      <c r="AM1" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="AN1" t="s">
+      <c r="AN1" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="AO1" t="s">
+      <c r="AO1" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="AP1" t="s">
+      <c r="AP1" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="AQ1" t="s">
+      <c r="AQ1" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="AR1" t="s">
+      <c r="AR1" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="AS1" t="s">
+      <c r="AS1" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="AT1" t="s">
+      <c r="AT1" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="AU1" t="s">
+      <c r="AU1" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="AV1" t="s">
+      <c r="AV1" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="AW1" t="s">
+      <c r="AW1" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="AX1" t="s">
+      <c r="AX1" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="AY1" t="s">
+      <c r="AY1" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="AZ1" t="s">
+      <c r="AZ1" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="BA1" t="s">
+      <c r="BA1" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="BB1" t="s">
+      <c r="BB1" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="BC1" t="s">
+      <c r="BC1" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="BD1" t="s">
+      <c r="BD1" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="BE1" t="s">
+      <c r="BE1" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="BF1" t="s">
+      <c r="BF1" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="BG1" t="s">
+      <c r="BG1" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="BH1" t="s">
+      <c r="BH1" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="BI1" t="s">
+      <c r="BI1" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="BJ1" t="s">
+      <c r="BJ1" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="BK1" t="s">
+      <c r="BK1" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="BL1" t="s">
+      <c r="BL1" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="BM1" t="s">
+      <c r="BM1" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="BN1" t="s">
+      <c r="BN1" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="BO1" t="s">
+      <c r="BO1" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="BP1" t="s">
+      <c r="BP1" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="BQ1" t="s">
+      <c r="BQ1" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="BR1" t="s">
+      <c r="BR1" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="BS1" t="s">
+      <c r="BS1" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="BT1" t="s">
+      <c r="BT1" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="BU1" t="s">
+      <c r="BU1" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="BV1" t="s">
+      <c r="BV1" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="BW1" t="s">
+      <c r="BW1" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="BX1" t="s">
+      <c r="BX1" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="BY1" t="s">
+      <c r="BY1" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="BZ1" t="s">
+      <c r="BZ1" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="CA1" t="s">
+      <c r="CA1" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="CB1" t="s">
+      <c r="CB1" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="CC1" t="s">
+      <c r="CC1" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="CD1" t="s">
+      <c r="CD1" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="CE1" t="s">
+      <c r="CE1" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="CF1" t="s">
+      <c r="CF1" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="CG1" t="s">
+      <c r="CG1" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="CH1" t="s">
+      <c r="CH1" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="CI1" t="s">
+      <c r="CI1" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="CJ1" t="s">
+      <c r="CJ1" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="CK1" t="s">
+      <c r="CK1" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="CL1" t="s">
+      <c r="CL1" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="CM1" t="s">
+      <c r="CM1" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="CN1" t="s">
+      <c r="CN1" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="CO1" t="s">
+      <c r="CO1" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="CP1" t="s">
+      <c r="CP1" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="CQ1" t="s">
+      <c r="CQ1" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="CR1" t="s">
+      <c r="CR1" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="CS1" t="s">
+      <c r="CS1" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="CT1" t="s">
+      <c r="CT1" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="CU1" t="s">
+      <c r="CU1" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="CV1" t="s">
+      <c r="CV1" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="CW1" t="s">
+      <c r="CW1" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="CX1" t="s">
+      <c r="CX1" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="CY1" t="s">
+      <c r="CY1" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="CZ1" t="s">
+      <c r="CZ1" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="DA1" t="s">
+      <c r="DA1" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="DB1" t="s">
+      <c r="DB1" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="DC1" t="s">
+      <c r="DC1" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="DD1" t="s">
+      <c r="DD1" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="DE1" t="s">
+      <c r="DE1" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="DF1" t="s">
+      <c r="DF1" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="DG1" t="s">
+      <c r="DG1" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="DH1" t="s">
+      <c r="DH1" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="DI1" t="s">
+      <c r="DI1" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="DJ1" t="s">
+      <c r="DJ1" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="DK1" t="s">
+      <c r="DK1" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="DL1" t="s">
+      <c r="DL1" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="DM1" t="s">
+      <c r="DM1" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="DN1" t="s">
+      <c r="DN1" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="DO1" t="s">
+      <c r="DO1" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="DP1" t="s">
+      <c r="DP1" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="DQ1" t="s">
+      <c r="DQ1" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="DR1" t="s">
+      <c r="DR1" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="DS1" t="s">
+      <c r="DS1" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="DT1" t="s">
+      <c r="DT1" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="DU1" t="s">
+      <c r="DU1" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="DV1" t="s">
+      <c r="DV1" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="DW1" t="s">
+      <c r="DW1" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="DX1" t="s">
+      <c r="DX1" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="DY1" t="s">
+      <c r="DY1" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="DZ1" t="s">
+      <c r="DZ1" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="EA1" t="s">
+      <c r="EA1" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="EB1" t="s">
+      <c r="EB1" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="EC1" t="s">
+      <c r="EC1" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="ED1" t="s">
+      <c r="ED1" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="EE1" t="s">
+      <c r="EE1" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="EF1" t="s">
+      <c r="EF1" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="EG1" t="s">
+      <c r="EG1" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="EH1" t="s">
+      <c r="EH1" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="EI1" t="s">
+      <c r="EI1" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="EJ1" t="s">
+      <c r="EJ1" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="EK1" t="s">
+      <c r="EK1" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="EL1" t="s">
+      <c r="EL1" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="EM1" t="s">
+      <c r="EM1" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="EN1" t="s">
+      <c r="EN1" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="EO1" t="s">
+      <c r="EO1" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="EP1" t="s">
+      <c r="EP1" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="EQ1" t="s">
+      <c r="EQ1" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="ER1" t="s">
+      <c r="ER1" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="ES1" t="s">
+      <c r="ES1" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="ET1" t="s">
+      <c r="ET1" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="EU1" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="EV1" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="EU1" t="s">
+      <c r="EW1" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="EV1" t="s">
+      <c r="EX1" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="EY1" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="EZ1" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="FA1" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="FB1" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="EW1" t="s">
+      <c r="FC1" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="EX1" t="s">
+      <c r="FD1" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="EY1" t="s">
+      <c r="FE1" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="EZ1" t="s">
+      <c r="FF1" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="FA1" t="s">
+      <c r="FG1" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="FB1" t="s">
+      <c r="FH1" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="FC1" t="s">
+      <c r="FI1" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="FD1" t="s">
+      <c r="FJ1" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="FE1" t="s">
+      <c r="FK1" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="FF1" t="s">
+      <c r="FL1" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="FG1" t="s">
+      <c r="FM1" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="FH1" t="s">
+      <c r="FN1" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="FI1" t="s">
+      <c r="FO1" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="FJ1" t="s">
+      <c r="FP1" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="FK1" t="s">
+      <c r="FQ1" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="FL1" t="s">
+      <c r="FR1" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="FM1" t="s">
+      <c r="FS1" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="FN1" t="s">
+      <c r="FT1" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="FO1" t="s">
+      <c r="FU1" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="FP1" t="s">
+      <c r="FV1" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="FQ1" t="s">
+      <c r="FW1" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="FR1" t="s">
+      <c r="FX1" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="FS1" t="s">
+      <c r="FY1" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="FT1" t="s">
+      <c r="FZ1" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="FU1" t="s">
+      <c r="GA1" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="FV1" t="s">
+      <c r="GB1" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="FW1" t="s">
+      <c r="GC1" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="FX1" t="s">
+      <c r="GD1" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="FY1" t="s">
+      <c r="GE1" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="FZ1" t="s">
+      <c r="GF1" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="GA1" t="s">
+      <c r="GG1" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="GB1" t="s">
+      <c r="GH1" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="GC1" t="s">
+      <c r="GI1" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="GD1" t="s">
+      <c r="GJ1" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="GK1" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="GL1" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="GE1" t="s">
+      <c r="GM1" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="GF1" t="s">
+      <c r="GN1" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="GG1" t="s">
+      <c r="GO1" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="GH1" t="s">
+      <c r="GP1" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="GI1" t="s">
+      <c r="GQ1" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="GJ1" t="s">
-        <v>191</v>
-      </c>
-      <c r="GK1" t="s">
-        <v>192</v>
-      </c>
-      <c r="GL1" t="s">
-        <v>193</v>
-      </c>
-      <c r="GM1" t="s">
-        <v>194</v>
-      </c>
-      <c r="GN1" t="s">
-        <v>195</v>
-      </c>
-      <c r="GO1" t="s">
-        <v>196</v>
-      </c>
-      <c r="GP1" t="s">
-        <v>197</v>
-      </c>
-      <c r="GQ1" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="2" spans="1:199" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:199">
       <c r="A2" s="1"/>
     </row>
-    <row r="3" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:199">
       <c r="A3" s="1"/>
     </row>
-    <row r="4" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:199">
       <c r="A4" s="1"/>
     </row>
-    <row r="5" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:199">
       <c r="A5" s="1"/>
     </row>
-    <row r="6" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:199">
       <c r="A6" s="1"/>
     </row>
-    <row r="7" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:199">
       <c r="A7" s="1"/>
     </row>
-    <row r="8" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:199">
       <c r="A8" s="1"/>
     </row>
-    <row r="9" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:199">
       <c r="A9" s="1"/>
     </row>
-    <row r="10" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:199">
       <c r="A10" s="1"/>
     </row>
-    <row r="11" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:199">
       <c r="A11" s="1"/>
     </row>
-    <row r="12" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:199">
       <c r="A12" s="1"/>
     </row>
-    <row r="13" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:199">
       <c r="A13" s="1"/>
     </row>
-    <row r="14" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:199">
       <c r="A14" s="1"/>
     </row>
-    <row r="15" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:199">
       <c r="A15" s="1"/>
     </row>
-    <row r="16" spans="1:199" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:199">
       <c r="A16" s="1"/>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:1">
       <c r="A17" s="1"/>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:1">
       <c r="A18" s="1"/>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:1">
       <c r="A19" s="1"/>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:1">
       <c r="A20" s="1"/>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:1">
       <c r="A21" s="1"/>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:1">
       <c r="A22" s="1"/>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:1">
       <c r="A23" s="1"/>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:1">
       <c r="A24" s="1"/>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:1">
       <c r="A25" s="1"/>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:1">
       <c r="A26" s="1"/>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:1">
       <c r="A27" s="1"/>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:1">
       <c r="A28" s="1"/>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:1">
       <c r="A29" s="1"/>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:1">
       <c r="A30" s="1"/>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:1">
       <c r="A31" s="1"/>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:1">
       <c r="A32" s="1"/>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:1">
       <c r="A33" s="1"/>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:1">
       <c r="A34" s="1"/>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:1">
       <c r="A35" s="1"/>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:1">
       <c r="A36" s="1"/>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:1">
       <c r="A37" s="1"/>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:1">
       <c r="A38" s="1"/>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:1">
       <c r="A39" s="1"/>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:1">
       <c r="A40" s="1"/>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:1">
       <c r="A41" s="1"/>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:1">
       <c r="A42" s="1"/>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:1">
       <c r="A43" s="1"/>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:1">
       <c r="A44" s="1"/>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:1">
       <c r="A45" s="1"/>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:1">
       <c r="A46" s="1"/>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:1">
       <c r="A47" s="1"/>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:1">
       <c r="A48" s="1"/>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:1">
       <c r="A49" s="1"/>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:1">
       <c r="A50" s="1"/>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:1">
       <c r="A51" s="1"/>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:1">
       <c r="A52" s="1"/>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:1">
       <c r="A53" s="1"/>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:1">
       <c r="A54" s="1"/>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:1">
       <c r="A55" s="1"/>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:1">
       <c r="A56" s="1"/>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:1">
       <c r="A57" s="1"/>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:1">
       <c r="A58" s="1"/>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:1">
       <c r="A59" s="1"/>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:1">
       <c r="A60" s="1"/>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:1">
       <c r="A61" s="1"/>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:1">
       <c r="A62" s="1"/>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:1">
       <c r="A63" s="1"/>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:1">
       <c r="A64" s="1"/>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:1">
       <c r="A65" s="1"/>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:1">
       <c r="A66" s="1"/>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:1">
       <c r="A67" s="1"/>
     </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:1">
       <c r="A68" s="1"/>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:1">
       <c r="A69" s="1"/>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:1">
       <c r="A70" s="1"/>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:1">
       <c r="A71" s="1"/>
     </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:1">
       <c r="A72" s="1"/>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:1">
       <c r="A73" s="1"/>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:1">
       <c r="A74" s="1"/>
     </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:1">
       <c r="A75" s="1"/>
     </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:1">
       <c r="A76" s="1"/>
     </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:1">
       <c r="A77" s="1"/>
     </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:1">
       <c r="A78" s="1"/>
     </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:1">
       <c r="A79" s="1"/>
     </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:1">
       <c r="A80" s="1"/>
     </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:1">
       <c r="A81" s="1"/>
     </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:1">
       <c r="A82" s="1"/>
     </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:1">
       <c r="A83" s="1"/>
     </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:1">
       <c r="A84" s="1"/>
     </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:1">
       <c r="A85" s="1"/>
     </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:1">
       <c r="A86" s="1"/>
     </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:1">
       <c r="A87" s="1"/>
     </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:1">
       <c r="A88" s="1"/>
     </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:1">
       <c r="A89" s="1"/>
     </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:1">
       <c r="A90" s="1"/>
     </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:1">
       <c r="A91" s="1"/>
     </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:1">
       <c r="A92" s="1"/>
     </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:1">
       <c r="A93" s="1"/>
     </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:1">
       <c r="A94" s="1"/>
     </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:1">
       <c r="A95" s="1"/>
     </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:1">
       <c r="A96" s="1"/>
     </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:1">
       <c r="A97" s="1"/>
     </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:1">
       <c r="A98" s="1"/>
     </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:1">
       <c r="A99" s="1"/>
     </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:1">
       <c r="A100" s="1"/>
     </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:1">
       <c r="A101" s="1"/>
     </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:1">
       <c r="A102" s="1"/>
     </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:1">
       <c r="A103" s="1"/>
     </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:1">
       <c r="A104" s="1"/>
     </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:1">
       <c r="A105" s="1"/>
     </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:1">
       <c r="A106" s="1"/>
     </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:1">
       <c r="A107" s="1"/>
     </row>
-    <row r="108" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:1">
       <c r="A108" s="1"/>
     </row>
-    <row r="109" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:1">
       <c r="A109" s="1"/>
     </row>
-    <row r="110" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:1">
       <c r="A110" s="1"/>
     </row>
-    <row r="111" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:1">
       <c r="A111" s="1"/>
     </row>
-    <row r="112" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:1">
       <c r="A112" s="1"/>
     </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:1">
       <c r="A113" s="1"/>
     </row>
-    <row r="114" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:1">
       <c r="A114" s="1"/>
     </row>
-    <row r="115" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:1">
       <c r="A115" s="1"/>
     </row>
-    <row r="116" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:1">
       <c r="A116" s="1"/>
     </row>
-    <row r="117" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:1">
       <c r="A117" s="1"/>
     </row>
-    <row r="118" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:1">
       <c r="A118" s="1"/>
     </row>
-    <row r="119" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:1">
       <c r="A119" s="1"/>
     </row>
-    <row r="120" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:1">
       <c r="A120" s="1"/>
     </row>
-    <row r="121" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:1">
       <c r="A121" s="1"/>
     </row>
-    <row r="122" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:1">
       <c r="A122" s="1"/>
     </row>
-    <row r="123" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:1">
       <c r="A123" s="1"/>
     </row>
-    <row r="124" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:1">
       <c r="A124" s="1"/>
     </row>
-    <row r="125" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:1">
       <c r="A125" s="1"/>
     </row>
-    <row r="126" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:1">
       <c r="A126" s="1"/>
     </row>
-    <row r="127" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:1">
       <c r="A127" s="1"/>
     </row>
-    <row r="128" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:1">
       <c r="A128" s="1"/>
     </row>
-    <row r="129" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:1">
       <c r="A129" s="1"/>
     </row>
-    <row r="130" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:1">
       <c r="A130" s="1"/>
     </row>
-    <row r="131" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:1">
       <c r="A131" s="1"/>
     </row>
-    <row r="132" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:1">
       <c r="A132" s="1"/>
     </row>
-    <row r="133" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:1">
       <c r="A133" s="1"/>
     </row>
-    <row r="134" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:1">
       <c r="A134" s="1"/>
     </row>
-    <row r="135" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:1">
       <c r="A135" s="1"/>
     </row>
-    <row r="136" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:1">
       <c r="A136" s="1"/>
     </row>
-    <row r="137" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:1">
       <c r="A137" s="1"/>
     </row>
-    <row r="138" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:1">
       <c r="A138" s="1"/>
     </row>
-    <row r="139" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:1">
       <c r="A139" s="1"/>
     </row>
-    <row r="140" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:1">
       <c r="A140" s="1"/>
     </row>
-    <row r="141" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:1">
       <c r="A141" s="1"/>
     </row>
-    <row r="142" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:1">
       <c r="A142" s="1"/>
     </row>
-    <row r="143" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:1">
       <c r="A143" s="1"/>
     </row>
-    <row r="144" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:1">
       <c r="A144" s="1"/>
     </row>
-    <row r="145" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:1">
       <c r="A145" s="1"/>
     </row>
-    <row r="146" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:1">
       <c r="A146" s="1"/>
     </row>
-    <row r="147" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:1">
       <c r="A147" s="1"/>
     </row>
-    <row r="148" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:1">
       <c r="A148" s="1"/>
     </row>
-    <row r="149" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:1">
       <c r="A149" s="1"/>
     </row>
-    <row r="150" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:1">
       <c r="A150" s="1"/>
     </row>
-    <row r="151" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:1">
       <c r="A151" s="1"/>
     </row>
-    <row r="152" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:1">
       <c r="A152" s="1"/>
     </row>
-    <row r="153" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:1">
       <c r="A153" s="1"/>
     </row>
-    <row r="154" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:1">
       <c r="A154" s="1"/>
     </row>
-    <row r="155" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:1">
       <c r="A155" s="1"/>
     </row>
-    <row r="156" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:1">
       <c r="A156" s="1"/>
     </row>
-    <row r="157" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:1">
       <c r="A157" s="1"/>
     </row>
-    <row r="158" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:1">
       <c r="A158" s="1"/>
     </row>
-    <row r="159" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:1">
       <c r="A159" s="1"/>
     </row>
-    <row r="160" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:1">
       <c r="A160" s="1"/>
     </row>
-    <row r="161" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:1">
       <c r="A161" s="1"/>
     </row>
-    <row r="162" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:1">
       <c r="A162" s="1"/>
     </row>
-    <row r="163" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:1">
       <c r="A163" s="1"/>
     </row>
-    <row r="164" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:1">
       <c r="A164" s="1"/>
     </row>
-    <row r="165" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:1">
       <c r="A165" s="1"/>
     </row>
-    <row r="166" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:1">
       <c r="A166" s="1"/>
     </row>
-    <row r="167" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:1">
       <c r="A167" s="1"/>
     </row>
-    <row r="168" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:1">
       <c r="A168" s="1"/>
     </row>
-    <row r="169" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:1">
       <c r="A169" s="1"/>
     </row>
-    <row r="170" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:1">
       <c r="A170" s="1"/>
     </row>
-    <row r="171" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:1">
       <c r="A171" s="1"/>
     </row>
-    <row r="172" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:1">
       <c r="A172" s="1"/>
     </row>
-    <row r="173" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:1">
       <c r="A173" s="1"/>
     </row>
-    <row r="174" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:1">
       <c r="A174" s="1"/>
     </row>
-    <row r="175" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:1">
       <c r="A175" s="1"/>
     </row>
-    <row r="176" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:1">
       <c r="A176" s="1"/>
     </row>
-    <row r="177" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:1">
       <c r="A177" s="1"/>
     </row>
-    <row r="178" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:1">
       <c r="A178" s="1"/>
     </row>
-    <row r="179" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:1">
       <c r="A179" s="1"/>
     </row>
-    <row r="180" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:1">
       <c r="A180" s="1"/>
     </row>
-    <row r="181" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:1">
       <c r="A181" s="1"/>
     </row>
-    <row r="182" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:1">
       <c r="A182" s="1"/>
     </row>
-    <row r="183" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:1">
       <c r="A183" s="1"/>
     </row>
-    <row r="184" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:1">
       <c r="A184" s="1"/>
     </row>
-    <row r="185" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:1">
       <c r="A185" s="1"/>
     </row>
-    <row r="186" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:1">
       <c r="A186" s="1"/>
     </row>
-    <row r="187" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:1">
       <c r="A187" s="1"/>
     </row>
-    <row r="188" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:1">
       <c r="A188" s="1"/>
     </row>
-    <row r="189" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:1">
       <c r="A189" s="1"/>
     </row>
-    <row r="190" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:1">
       <c r="A190" s="1"/>
     </row>
-    <row r="191" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:1">
       <c r="A191" s="1"/>
     </row>
-    <row r="192" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:1">
       <c r="A192" s="1"/>
     </row>
-    <row r="193" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:1">
       <c r="A193" s="1"/>
     </row>
-    <row r="194" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:1">
       <c r="A194" s="1"/>
     </row>
-    <row r="195" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:1">
       <c r="A195" s="1"/>
     </row>
-    <row r="196" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:1">
       <c r="A196" s="1"/>
     </row>
-    <row r="197" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:1">
       <c r="A197" s="1"/>
     </row>
-    <row r="198" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:1">
       <c r="A198" s="1"/>
     </row>
-    <row r="199" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:1">
       <c r="A199" s="1"/>
     </row>
   </sheetData>

</xml_diff>